<commit_message>
update project and excel data
</commit_message>
<xml_diff>
--- a/data/ISO 27001 Maturity Assessments 2027.xlsx
+++ b/data/ISO 27001 Maturity Assessments 2027.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kone-my.sharepoint.com/personal/syedarabia_basri_kone_com/Documents/Documents/getting-started-sample - Copy/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kone-my.sharepoint.com/personal/syedarabia_basri_kone_com/Documents/Documents/getting-started-sample - Copy/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{61C8D642-53A3-43C5-B1D6-51A7B2325C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="92" documentId="8_{61C8D642-53A3-43C5-B1D6-51A7B2325C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6F7F693-2513-4143-A8EE-0FDD1995A8E9}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{09EAD548-590F-42CA-9C1D-B19970AFC76D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{09EAD548-590F-42CA-9C1D-B19970AFC76D}"/>
   </bookViews>
   <sheets>
     <sheet name="HR Security Maturity" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="215">
   <si>
     <t>Category</t>
   </si>
@@ -386,13 +386,323 @@
   </si>
   <si>
     <t>5.23.3 Information security for use of cloud services</t>
+  </si>
+  <si>
+    <t>Czechia ISO 27001</t>
+  </si>
+  <si>
+    <t>UAE ISO 27001</t>
+  </si>
+  <si>
+    <t>Netherlands ISO 27001</t>
+  </si>
+  <si>
+    <t>Germany ISO 27001</t>
+  </si>
+  <si>
+    <t>Malaysia ISO 27001</t>
+  </si>
+  <si>
+    <t>Austria ISO 27001</t>
+  </si>
+  <si>
+    <t>Canada ISO 27001</t>
+  </si>
+  <si>
+    <t>Belgium ISO 27001</t>
+  </si>
+  <si>
+    <t>France ISO 27001</t>
+  </si>
+  <si>
+    <t>Australia ISO 27001</t>
+  </si>
+  <si>
+    <t>Bulgaria ISO 27001</t>
+  </si>
+  <si>
+    <t>Slovakia ISO 27001</t>
+  </si>
+  <si>
+    <t>7.12.1 Cabling security</t>
+  </si>
+  <si>
+    <t>Power and telecommunications lines in the information processing facilities must be underground, where possible, or subject to adequate alternative protection.</t>
+  </si>
+  <si>
+    <t>7.12.2 Cabling security</t>
+  </si>
+  <si>
+    <t>Network cabling must be protected from unauthorized interception or damage, for example by using conduit or by avoiding routes through public areas.</t>
+  </si>
+  <si>
+    <t>7.12.3 Cabling security</t>
+  </si>
+  <si>
+    <t>Power cables must be segregated from communications cables to prevent interference.</t>
+  </si>
+  <si>
+    <t>8.1 User endpoint devices</t>
+  </si>
+  <si>
+    <t>All desktop and laptop hard disks are encrypted according to the Information Security policy</t>
+  </si>
+  <si>
+    <t>7.7 Clear desk and clear screen</t>
+  </si>
+  <si>
+    <t>All desktops, laptops and terminals are signed out or screen locked when unattended</t>
+  </si>
+  <si>
+    <t>7.8.1 Equipment siting and protection</t>
+  </si>
+  <si>
+    <t>Printers sited in a way that they cannot be accessed by unauthorized people</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.5.1 Protecting against physical and environmental threats </t>
+  </si>
+  <si>
+    <t>Intrusion detection system with an alarm</t>
+  </si>
+  <si>
+    <t>7.5.2 Protecting against physical and environmental threats</t>
+  </si>
+  <si>
+    <t>Automatic fire indication system</t>
+  </si>
+  <si>
+    <t>7.5.3 Protecting against physical and environmental threats</t>
+  </si>
+  <si>
+    <t>Portable fire extinguisher</t>
+  </si>
+  <si>
+    <t>7.5.4 Protecting against physical and environmental threats</t>
+  </si>
+  <si>
+    <t>Emergency illumination and exit</t>
+  </si>
+  <si>
+    <t>7.5.5 Protecting against physical and environmental threats</t>
+  </si>
+  <si>
+    <t>security lighting</t>
+  </si>
+  <si>
+    <t>7.13.1 Equipment maintenance</t>
+  </si>
+  <si>
+    <t>The above control systems must be maintained and checked regularly according to manufacturers’ instructions and local legislation.</t>
+  </si>
+  <si>
+    <t>5.12 Classification of information</t>
+  </si>
+  <si>
+    <t>In case an employee works from a home office or outside KONE premises, KONE business critical and sensitive information must be stored in accordance with the Information Security Policy (Policy-0075).</t>
+  </si>
+  <si>
+    <t>7.2.1 Physical entry controls</t>
+  </si>
+  <si>
+    <t>KONE standard ID badges visibly used by KONE employees, contractors, temporary workers and visitors. When granting the physical access rights (e.g. KONE ID Badges or separate tokens) to new employees or providing temporary access cards, the identity of the recipient must be verified.</t>
+  </si>
+  <si>
+    <t>8.20 Networks security</t>
+  </si>
+  <si>
+    <t>Any network functionalities are centrally managed by KONE IT.</t>
+  </si>
+  <si>
+    <t>7.2.2 Physical entry controls</t>
+  </si>
+  <si>
+    <t>Internal locking system and key management.
+o There must be a named KONE employee in charge of granting/revoking access rights and keys. Locking system should be such that the access keys cannot be duplicated without authorization from the KONE employee in charge of granting/revoking access rights and keys.
+o Access control rights and keys for each user of a group must be based on work duties and granted for a defined time period. Temporary access rights and keys must be authorized by a KONE employee hosting the visitor.
+o Keys, access rights and other company property must be revoked and collected immediately after expiration of employment and when a person no longer has a valid business reason to enter the area in question;</t>
+  </si>
+  <si>
+    <t>7.4.1 Physical security monitoring</t>
+  </si>
+  <si>
+    <t>Intrusion detection system with alarm transmission to local KONE Call Center or to external service provider;</t>
+  </si>
+  <si>
+    <t>7.2.3 Physical entry controls</t>
+  </si>
+  <si>
+    <t>Access control system;</t>
+  </si>
+  <si>
+    <t>6.6 Confidentiality or non-disclosure agreements</t>
+  </si>
+  <si>
+    <t>KONE personnel, external service providers and visitors granted unsupervised access to Advanced Security Areas must sign a Non-Disclosure Agreement;</t>
+  </si>
+  <si>
+    <t>7.2.4 Physical entry controls</t>
+  </si>
+  <si>
+    <t>Visitors must be accompanied by a KONE host at all times and photographing is not allowed;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.4.2 Physical security monitoring </t>
+  </si>
+  <si>
+    <t>Camera monitoring system covering all entrances, exits and sensitive areas;</t>
+  </si>
+  <si>
+    <t>7.5.6 Protecting against physical and environmental threats</t>
+  </si>
+  <si>
+    <t>Uninterrupted Power Supply (UPS) system which provides power supply for critical detection, access control and alarm systems for at least 2 hours.</t>
+  </si>
+  <si>
+    <t>8.3 Information access restriction</t>
+  </si>
+  <si>
+    <t>Confidential information is stored in a secure place, such as designated locked cabinets, rooms or areas;</t>
+  </si>
+  <si>
+    <t>5.10 Acceptable use of information and other associated assets</t>
+  </si>
+  <si>
+    <t>There are documented rules for handling and disposal of sensitive documents and electronic data stored in hard drives in accordance with the Information Security Policy (Policy-0075);</t>
+  </si>
+  <si>
+    <t>6.1 Screening</t>
+  </si>
+  <si>
+    <t>-The need for pre-screening of employees must be considered based on Personnel Security guidelines;</t>
+  </si>
+  <si>
+    <t>6.3 Information security awareness, education and training</t>
+  </si>
+  <si>
+    <t>Relevant personnel must be sufficiently trained and made aware of the requirements and controls related to working in High Security Areas.</t>
+  </si>
+  <si>
+    <t>7.2.5 Physical entry controls</t>
+  </si>
+  <si>
+    <t>Local Owner is responsible for arranging the key and access management. The local Sponsor must authorize principles for providing access rights;</t>
+  </si>
+  <si>
+    <t>7.2.6 Physical entry controls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identification badge with photo and KONE logo visible at all times;
+</t>
+  </si>
+  <si>
+    <t>7.2.7 Physical entry controls</t>
+  </si>
+  <si>
+    <t>-Access control system capable of providing audit trail on entry events;</t>
+  </si>
+  <si>
+    <t>7.2.8 Physical entry controls</t>
+  </si>
+  <si>
+    <t>Physical access control system with PIN code or biometric readers. The access control system shall be designed so that each person seeking entry has valid access rights and knows a valid personal identification number or possesses the proper unique physical characteristics (e.g. fingerprint). The PIN code or biometric readers are active at minimum during outside of office hours. The access control system must be able to provide minimum 6 months history data on all access activity;</t>
+  </si>
+  <si>
+    <t>7.4.3 Physical security monitoring</t>
+  </si>
+  <si>
+    <t>Camera monitoring system with minimum 3 months recording and remote viewing capability to identify people covering all entrances, exits and sensitive areas;</t>
+  </si>
+  <si>
+    <t>7.4.4 Physical security monitoring</t>
+  </si>
+  <si>
+    <t>Patrol guarding and alarm response personnel must be applied. Patrolling is limited to perimeter walls, doors and windows of High Security Areas. The alarm response personnel are allowed to enter a High Security Area only if an alarm has gone off in such area;</t>
+  </si>
+  <si>
+    <t>7.3 Securing offices, rooms and facilities</t>
+  </si>
+  <si>
+    <t>Cleaning, maintenance, renovation and other similar works are to be carried out during office hours or in supervised conditions only. Access to be limited only to premises where such work is carried out. Generic access rights, such as master keys, to the premises and codes for intrusion detection systems cannot be provided to external parties;</t>
+  </si>
+  <si>
+    <t>7.1 Physical security perimeter</t>
+  </si>
+  <si>
+    <t>Fencing (applied to R&amp;D testing facilities, reliability laboratories and factories with AEO, C-TPAT or another similar license). The areas shall be fenced. Camera monitoring system with remote viewing capabilities that allow the site’s security personnel to observe the perimeter fencing;</t>
+  </si>
+  <si>
+    <t>7.8.2 Equipment siting and protection</t>
+  </si>
+  <si>
+    <t>Computing equipment is sited and protected to reduce risks from power failures, environmental threats and hazards, and opportunities for unauthorized access.</t>
+  </si>
+  <si>
+    <t>7.5.7 Protecting against physical and environmental threats</t>
+  </si>
+  <si>
+    <t>Separate cooling</t>
+  </si>
+  <si>
+    <t>7.5.8 Protecting against physical and environmental threats</t>
+  </si>
+  <si>
+    <t>Redundant power circuits:
+o one for the UPS power
+o one for the dirty power
+o disconnects for each rack located in the data room</t>
+  </si>
+  <si>
+    <t>7.2.9 Physical entry controls</t>
+  </si>
+  <si>
+    <t>Badge access for authorized personnel only</t>
+  </si>
+  <si>
+    <t>7.2.10 Physical entry controls</t>
+  </si>
+  <si>
+    <t>Building access process to be setup for suppliers outside of the business hours</t>
+  </si>
+  <si>
+    <t>7.5.9 Protecting against physical and environmental threats </t>
+  </si>
+  <si>
+    <t>Anti-static flooring</t>
+  </si>
+  <si>
+    <t>7.5.10 Protecting against physical and environmental threats </t>
+  </si>
+  <si>
+    <t>Redundant cooling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.5.11 Protecting against physical and environmental threats </t>
+  </si>
+  <si>
+    <t>-Conditioned Power: Generator &amp; UPS</t>
+  </si>
+  <si>
+    <t>7.5.12 Protecting against physical and environmental threats </t>
+  </si>
+  <si>
+    <t>Fire Suppression</t>
+  </si>
+  <si>
+    <t>7.5.13 Protecting against physical and environmental threats</t>
+  </si>
+  <si>
+    <t>Temperature and humidity monitoring</t>
+  </si>
+  <si>
+    <t>7.13.2 Equipment maintenance</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -424,6 +734,18 @@
       <name val="Segoe UI"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF333333"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -445,7 +767,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -459,6 +781,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -793,19 +1119,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C71DA111-6A29-426B-AA7D-B2135B3CADD6}">
-  <dimension ref="A1:G23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:S23"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="67.28515625" customWidth="1"/>
-    <col min="2" max="2" width="76.42578125" customWidth="1"/>
-    <col min="3" max="3" width="40" customWidth="1"/>
-    <col min="4" max="4" width="41.85546875" customWidth="1"/>
-    <col min="5" max="5" width="74.28515625" customWidth="1"/>
-    <col min="6" max="6" width="67.7109375" customWidth="1"/>
-    <col min="7" max="7" width="71.7109375" customWidth="1"/>
+    <col min="1" max="1" width="67.26953125" customWidth="1"/>
+    <col min="2" max="2" width="76.453125" customWidth="1"/>
+    <col min="3" max="3" width="23.81640625" customWidth="1"/>
+    <col min="4" max="4" width="23" customWidth="1"/>
+    <col min="5" max="5" width="19.90625" customWidth="1"/>
+    <col min="6" max="6" width="20.36328125" customWidth="1"/>
+    <col min="7" max="7" width="16.6328125" customWidth="1"/>
+    <col min="8" max="8" width="21.453125" customWidth="1"/>
+    <col min="9" max="9" width="15.1796875" customWidth="1"/>
+    <col min="10" max="10" width="21.1796875" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="17.1796875" customWidth="1"/>
+    <col min="13" max="13" width="17.7265625" customWidth="1"/>
+    <col min="14" max="14" width="16.453125" customWidth="1"/>
+    <col min="15" max="15" width="16.6328125" customWidth="1"/>
+    <col min="16" max="16" width="15.1796875" customWidth="1"/>
+    <col min="17" max="17" width="17.90625" customWidth="1"/>
+    <col min="18" max="18" width="20.6328125" customWidth="1"/>
+    <col min="19" max="19" width="18.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -827,8 +1165,44 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H1" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="N1" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="O1" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="P1" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q1" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="R1" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="S1" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -836,7 +1210,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>9</v>
       </c>
@@ -844,7 +1218,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
@@ -852,7 +1226,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
@@ -860,7 +1234,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
@@ -868,7 +1242,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>17</v>
       </c>
@@ -876,7 +1250,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>19</v>
       </c>
@@ -884,7 +1258,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>21</v>
       </c>
@@ -892,7 +1266,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -900,7 +1274,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -908,7 +1282,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -916,7 +1290,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>29</v>
       </c>
@@ -924,7 +1298,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>31</v>
       </c>
@@ -932,7 +1306,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -940,7 +1314,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -948,7 +1322,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>37</v>
       </c>
@@ -956,7 +1330,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -964,7 +1338,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -972,7 +1346,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>43</v>
       </c>
@@ -980,7 +1354,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>45</v>
       </c>
@@ -988,7 +1362,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>47</v>
       </c>
@@ -996,7 +1370,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>49</v>
       </c>
@@ -1014,20 +1388,31 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7D8E7A6-C0BE-4006-B921-A4F2817013BC}">
-  <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:S12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="37" customWidth="1"/>
     <col min="2" max="2" width="54" customWidth="1"/>
-    <col min="3" max="3" width="25.7109375" customWidth="1"/>
-    <col min="4" max="4" width="28.140625" customWidth="1"/>
-    <col min="5" max="5" width="26.28515625" customWidth="1"/>
-    <col min="6" max="6" width="29" customWidth="1"/>
-    <col min="7" max="7" width="29.140625" customWidth="1"/>
-    <col min="8" max="8" width="18.85546875" customWidth="1"/>
+    <col min="3" max="3" width="25.7265625" customWidth="1"/>
+    <col min="4" max="4" width="28.1796875" customWidth="1"/>
+    <col min="5" max="5" width="26.26953125" customWidth="1"/>
+    <col min="6" max="6" width="21.6328125" customWidth="1"/>
+    <col min="7" max="7" width="15.90625" customWidth="1"/>
+    <col min="8" max="8" width="18.81640625" customWidth="1"/>
+    <col min="9" max="9" width="16.7265625" customWidth="1"/>
+    <col min="10" max="10" width="20.81640625" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" customWidth="1"/>
+    <col min="12" max="12" width="18.26953125" customWidth="1"/>
+    <col min="13" max="13" width="19.36328125" customWidth="1"/>
+    <col min="14" max="14" width="19.1796875" customWidth="1"/>
+    <col min="15" max="15" width="18.81640625" customWidth="1"/>
+    <col min="16" max="16" width="17.453125" customWidth="1"/>
+    <col min="17" max="17" width="17.54296875" customWidth="1"/>
+    <col min="18" max="18" width="18" customWidth="1"/>
+    <col min="19" max="19" width="18.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1049,8 +1434,44 @@
       <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="255" x14ac:dyDescent="0.25">
+      <c r="H1" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="N1" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="P1" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q1" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="R1" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="S1" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>51</v>
       </c>
@@ -1058,7 +1479,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="165" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>53</v>
       </c>
@@ -1066,7 +1487,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="225" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>55</v>
       </c>
@@ -1074,7 +1495,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="255" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>57</v>
       </c>
@@ -1082,7 +1503,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="180" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>59</v>
       </c>
@@ -1090,7 +1511,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="375" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>61</v>
       </c>
@@ -1098,7 +1519,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="195" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>63</v>
       </c>
@@ -1106,7 +1527,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="375.75" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" ht="73.5" x14ac:dyDescent="0.45">
       <c r="A9" s="5" t="s">
         <v>65</v>
       </c>
@@ -1114,7 +1535,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="240.75" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" ht="52.5" x14ac:dyDescent="0.45">
       <c r="A10" s="5" t="s">
         <v>67</v>
       </c>
@@ -1122,7 +1543,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="240" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>69</v>
       </c>
@@ -1130,7 +1551,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="300" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>71</v>
       </c>
@@ -1148,22 +1569,75 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BC43EF7-60AA-4577-A527-49300830E2DD}">
-  <dimension ref="A1:B22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:S22"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="47.5703125" customWidth="1"/>
-    <col min="2" max="2" width="84.7109375" customWidth="1"/>
+    <col min="1" max="1" width="47.54296875" customWidth="1"/>
+    <col min="2" max="2" width="84.7265625" customWidth="1"/>
+    <col min="3" max="3" width="17.08984375" customWidth="1"/>
+    <col min="19" max="19" width="16.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="240" x14ac:dyDescent="0.25">
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="N1" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="O1" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="P1" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q1" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="R1" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="S1" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>93</v>
       </c>
@@ -1171,7 +1645,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="135" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>94</v>
       </c>
@@ -1179,7 +1653,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>95</v>
       </c>
@@ -1187,7 +1661,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="195" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1195,7 +1669,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="255" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>97</v>
       </c>
@@ -1203,7 +1677,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="210" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>98</v>
       </c>
@@ -1211,7 +1685,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="150" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>99</v>
       </c>
@@ -1219,7 +1693,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="150" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>100</v>
       </c>
@@ -1227,7 +1701,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="195" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>101</v>
       </c>
@@ -1235,7 +1709,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="225" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>102</v>
       </c>
@@ -1243,7 +1717,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="225" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>103</v>
       </c>
@@ -1251,7 +1725,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="345" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>104</v>
       </c>
@@ -1259,7 +1733,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="225" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>105</v>
       </c>
@@ -1267,7 +1741,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="165" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>106</v>
       </c>
@@ -1275,7 +1749,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="195" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>107</v>
       </c>
@@ -1283,7 +1757,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="270" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>108</v>
       </c>
@@ -1291,7 +1765,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="210" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>109</v>
       </c>
@@ -1299,7 +1773,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="195" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>110</v>
       </c>
@@ -1307,7 +1781,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="300" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>111</v>
       </c>
@@ -1315,7 +1789,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="360" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>112</v>
       </c>
@@ -1323,7 +1797,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="225" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>113</v>
       </c>
@@ -1341,9 +1815,433 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0614127-D2DF-4B83-A42C-98228CA9F683}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <dimension ref="A1:S46"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="30.81640625" customWidth="1"/>
+    <col min="2" max="2" width="50.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="N1" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="O1" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="P1" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q1" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="R1" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="S1" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="58" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>134</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>136</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B8" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B9" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B11" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B12" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="58" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>148</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="87" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>150</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" ht="116" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>152</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>154</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="319" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>156</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>158</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>160</v>
+      </c>
+      <c r="B19" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>164</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>166</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>170</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>174</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="59" x14ac:dyDescent="0.45">
+      <c r="A27" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>178</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>180</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>182</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>184</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="116" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A36" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A37" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B37" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="B41" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B42" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B43" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B44" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B45" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>214</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddHeader>&amp;R&amp;"arial"&amp;8&amp;K000000 KONE Internal&amp;1#_x000D_</oddHeader>
@@ -1354,7 +2252,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D8ABF13-6D36-4C8F-B396-DCCCD72099B9}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>